<commit_message>
ajuste de dados 03-08-2026
</commit_message>
<xml_diff>
--- a/finalData.xlsx
+++ b/finalData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://touticosmeticsbr-my.sharepoint.com/personal/rubens_pereira_kioskbrands_com/Documents/Documents/Touti-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{51540507-6717-4395-99D0-23A9EF8DE568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0891B653-C170-43A0-BD82-4F774950E61E}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{51540507-6717-4395-99D0-23A9EF8DE568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{062E51A4-AE52-4D6E-B11A-308A8C1DE081}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10178" uniqueCount="5574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10182" uniqueCount="5576">
   <si>
     <t>NOME FANTASIA</t>
   </si>
@@ -16766,6 +16766,12 @@
   </si>
   <si>
     <t>-23.22261761091795</t>
+  </si>
+  <si>
+    <t>-16.465159128892907</t>
+  </si>
+  <si>
+    <t>-54.62973075033013</t>
   </si>
 </sst>
 </file>
@@ -17009,7 +17015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -17136,6 +17142,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -64215,6 +64224,19 @@
       <c r="P915" s="13" t="s">
         <v>5571</v>
       </c>
+      <c r="Q915" s="13" t="s">
+        <v>5574</v>
+      </c>
+      <c r="R915" s="13" t="s">
+        <v>5575</v>
+      </c>
+      <c r="S915" s="54"/>
+      <c r="T915" s="13" t="s">
+        <v>5574</v>
+      </c>
+      <c r="U915" s="13" t="s">
+        <v>5575</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U594" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>